<commit_message>
Update help_config.json to clarify 'new' command description
</commit_message>
<xml_diff>
--- a/Data/Assertion_TF.xlsx
+++ b/Data/Assertion_TF.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29318"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://oneharman-my.sharepoint.com/personal/sophia_kim_harman_com/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://oneharman-my.sharepoint.com/personal/junsik_choi_harman_com/Documents/문서/TF자료/Assertion TF/Assertion Script/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2372" documentId="8_{1594ECDE-2767-4759-96A7-6FE2F184C525}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{45EF610C-9EF8-4AC6-B71E-9AD4DCB187A2}"/>
+  <xr:revisionPtr revIDLastSave="2373" documentId="8_{1594ECDE-2767-4759-96A7-6FE2F184C525}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{91F4ED20-E562-4B49-A219-AF0D2E163B48}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="5070" windowWidth="29040" windowHeight="15720" firstSheet="4" activeTab="2" xr2:uid="{A0D018F4-3A48-4DCB-A1A2-EA6BF4E4311F}"/>
+    <workbookView xWindow="-28800" yWindow="5535" windowWidth="38700" windowHeight="15345" xr2:uid="{A0D018F4-3A48-4DCB-A1A2-EA6BF4E4311F}"/>
   </bookViews>
   <sheets>
     <sheet name="Define" sheetId="9" r:id="rId1"/>
@@ -55,9 +55,9 @@
   <commentList>
     <comment ref="I3" authorId="0" shapeId="0" xr:uid="{372E79E2-B979-45EA-A3D7-4E90DC8A7E1F}">
       <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t>[스레드 댓글]
+사용 중인 버전의 Excel에서 이 스레드 댓글을 읽을 수 있지만 파일을 이후 버전의 Excel에서 열면 편집 내용이 모두 제거됩니다. 자세한 정보: https://go.microsoft.com/fwlink/?linkid=870924.
+댓글:
     승훈님 좋습니다!!</t>
       </text>
     </comment>
@@ -75,38 +75,38 @@
   <commentList>
     <comment ref="B4" authorId="0" shapeId="0" xr:uid="{11F28A3C-C90D-4418-BB46-9B6DADCDBE4E}">
       <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t>[스레드 댓글]
+사용 중인 버전의 Excel에서 이 스레드 댓글을 읽을 수 있지만 파일을 이후 버전의 Excel에서 열면 편집 내용이 모두 제거됩니다. 자세한 정보: https://go.microsoft.com/fwlink/?linkid=870924.
+댓글:
     Default를 Posedge로 가정하는 것은 어떻게 생각하시나요
-Reply:
+답글:
     좋아요</t>
       </text>
     </comment>
     <comment ref="C4" authorId="1" shapeId="0" xr:uid="{EAEF4952-1559-4391-A03C-03F57B7ADC3C}">
       <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t>[스레드 댓글]
+사용 중인 버전의 Excel에서 이 스레드 댓글을 읽을 수 있지만 파일을 이후 버전의 Excel에서 열면 편집 내용이 모두 제거됩니다. 자세한 정보: https://go.microsoft.com/fwlink/?linkid=870924.
+댓글:
     사실 Clock도 왠만하면 한 IP나 블록에서 동일한 것을 사용할 것 같은데 따로 만든 이유는 Clock 대신 sync signal 같은거 활용하기 위함인가요?
 만약 그렇지 않다면 blk로 들어오는 main clock으로 고정하고 이 칸 간소화 가능할 것 같아요
-Reply:
+답글:
     rx assertion 보니까, clk을 base clk만 사용하지 않더라구요
-Reply:
+답글:
     그럼 유지해야겠군요 확인 감사합니다.</t>
       </text>
     </comment>
     <comment ref="G4" authorId="2" shapeId="0" xr:uid="{066F6494-15CB-41D2-A5E8-F35BD8460361}">
       <text>
-        <t xml:space="preserve">[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t xml:space="preserve">[스레드 댓글]
+사용 중인 버전의 Excel에서 이 스레드 댓글을 읽을 수 있지만 파일을 이후 버전의 Excel에서 열면 편집 내용이 모두 제거됩니다. 자세한 정보: https://go.microsoft.com/fwlink/?linkid=870924.
+댓글:
     |-&gt; 이거로 통일해 버리면 칸 하나 줄일 수 있을 것 같은데 어떻게 생각하시나요?
-Reply:
+답글:
     오케이~
-Reply:
+답글:
     ㅋㅋㅋㅋㅋ갑자기 다빈님이 전자과에 가게된 스토리가 오버랩되는데
-Reply:
+답글:
     일할땐 생각해요ㅋㅋㅋㅋㅋㅋㅋㅋㅋㅋㅋㅋㅋㅋ
 </t>
       </text>
@@ -125,38 +125,38 @@
   <commentList>
     <comment ref="B4" authorId="0" shapeId="0" xr:uid="{A5EE3683-DAAF-4AD0-95D0-B34E9981B26B}">
       <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t>[스레드 댓글]
+사용 중인 버전의 Excel에서 이 스레드 댓글을 읽을 수 있지만 파일을 이후 버전의 Excel에서 열면 편집 내용이 모두 제거됩니다. 자세한 정보: https://go.microsoft.com/fwlink/?linkid=870924.
+댓글:
     Default를 Posedge로 가정하는 것은 어떻게 생각하시나요
-Reply:
+답글:
     좋아요</t>
       </text>
     </comment>
     <comment ref="C4" authorId="1" shapeId="0" xr:uid="{FBABEDF7-5267-49E5-B5C6-B213E24A5F77}">
       <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t>[스레드 댓글]
+사용 중인 버전의 Excel에서 이 스레드 댓글을 읽을 수 있지만 파일을 이후 버전의 Excel에서 열면 편집 내용이 모두 제거됩니다. 자세한 정보: https://go.microsoft.com/fwlink/?linkid=870924.
+댓글:
     사실 Clock도 왠만하면 한 IP나 블록에서 동일한 것을 사용할 것 같은데 따로 만든 이유는 Clock 대신 sync signal 같은거 활용하기 위함인가요?
 만약 그렇지 않다면 blk로 들어오는 main clock으로 고정하고 이 칸 간소화 가능할 것 같아요
-Reply:
+답글:
     rx assertion 보니까, clk을 base clk만 사용하지 않더라구요
-Reply:
+답글:
     그럼 유지해야겠군요 확인 감사합니다.</t>
       </text>
     </comment>
     <comment ref="G4" authorId="2" shapeId="0" xr:uid="{AB18BE64-54B0-4373-A63D-1F608B3F50E6}">
       <text>
-        <t xml:space="preserve">[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t xml:space="preserve">[스레드 댓글]
+사용 중인 버전의 Excel에서 이 스레드 댓글을 읽을 수 있지만 파일을 이후 버전의 Excel에서 열면 편집 내용이 모두 제거됩니다. 자세한 정보: https://go.microsoft.com/fwlink/?linkid=870924.
+댓글:
     |-&gt; 이거로 통일해 버리면 칸 하나 줄일 수 있을 것 같은데 어떻게 생각하시나요?
-Reply:
+답글:
     오케이~
-Reply:
+답글:
     ㅋㅋㅋㅋㅋ갑자기 다빈님이 전자과에 가게된 스토리가 오버랩되는데
-Reply:
+답글:
     일할땐 생각해요ㅋㅋㅋㅋㅋㅋㅋㅋㅋㅋㅋㅋㅋㅋ
 </t>
       </text>
@@ -4677,7 +4677,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="표준" xfId="0" builtinId="0"/>
     <cellStyle name="표준 2" xfId="1" xr:uid="{BB1E0E6C-DA0D-43B5-A5C3-94756A668AC2}"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -5096,7 +5096,7 @@
   <sheetPr>
     <tabColor theme="5" tint="0.39997558519241921"/>
   </sheetPr>
-  <dimension ref="B1:N10"/>
+  <dimension ref="B1:N9"/>
   <sheetFormatPr defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="9" style="53"/>
@@ -5279,11 +5279,6 @@
       </c>
       <c r="N9" s="64" t="s">
         <v>13</v>
-      </c>
-    </row>
-    <row r="10" spans="2:14">
-      <c r="F10" s="55">
-        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -8891,7 +8886,7 @@
       <c r="AP20" s="74"/>
       <c r="AQ20" s="74"/>
     </row>
-    <row r="21" spans="2:43" ht="18.75">
+    <row r="21" spans="2:43" ht="20.25">
       <c r="B21"/>
       <c r="I21" s="113" t="s">
         <v>70</v>
@@ -9439,7 +9434,7 @@
     <row r="43" spans="2:19">
       <c r="B43"/>
     </row>
-    <row r="44" spans="2:19" ht="18.75">
+    <row r="44" spans="2:19" ht="20.25">
       <c r="B44"/>
       <c r="I44" s="113" t="s">
         <v>72</v>

</xml_diff>